<commit_message>
docs(aidlc): simplify 'What is covered' wording in the merged AIDLC sheet
Co-Authored-By: samrat.kar@infosys.com <samrat.kar@infosys.com>
</commit_message>
<xml_diff>
--- a/docs/migration/DEVIN-AIDLC-ACU-metrics-v2.xlsx
+++ b/docs/migration/DEVIN-AIDLC-ACU-metrics-v2.xlsx
@@ -573,7 +573,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="110" customHeight="1">
+    <row r="6" ht="62" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Inception</t>
@@ -619,11 +619,11 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Read package.json, angular.json, tsconfig*.json and the src/app tree; produced the migration BRD (current vs target versions, every breaking change 9-&gt;20); split it into units of work with acceptance criteria per unit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="110" customHeight="1">
+          <t>Understood the existing app and planned the migration: BRD of current vs target versions and every breaking change, broken into one unit of work per version with acceptance criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="62" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Construction</t>
@@ -669,11 +669,11 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>11 sequential major upgrades (ng update 9-&gt;10-&gt;...-&gt;20) with npm install + build + test after each; RxJS 6-&gt;7 and removal of rxjs-compat; Sass math.div fix; TSLint/codelyzer replaced by angular-eslint and all violations fixed; Protractor removed and Playwright e2e added; full standalone conversion (NgModules pruned, bootstrapApplication + provideRouter/provideServiceWorker); control-flow syntax (@if/@for) and inject() migration; new @angular/build:application builder; first unit specs written (repo had none); ops config updated (.travis.yml, firebase.json, ngsw-config.json, README). INCLUDES Operation (PR #35 raised, 0.5525 ACUs) and Validation (production build, service-worker and manifest served over HTTP, adversarial test plan, browser-testing handoff, 5.6204 ACUs).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="110" customHeight="1">
+          <t>Did the migration: 11 major Angular upgrades one at a time, modernised the code and toolchain (RxJS 7, ESLint, standalone, new control flow, new builder, Playwright tests) and updated the CI, hosting and docs config. Includes Operation (raised PR #35) and Validation (builds, lint, unit and e2e tests green after each step).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="62" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Governance / AIDLC tooling (optional)</t>
@@ -719,7 +719,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Not required to migrate the app. Byte-stable prompt-prefix generator (scripts/aidlc-prompt-prefix.mjs) that keeps the cached prefix identical across tasks, the AIDLC cost scripts, and the unit-status bookkeeping. One-time asset: reusable by every future migration, so it should be amortised, not charged to this migration.</t>
+          <t>Optional. Reusable AIDLC instrumentation - the stable prompt prefix and the cost/usage reporting scripts. Not needed to migrate the app, and reusable on future migrations.</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>What the migration itself cost if the reusable AIDLC tooling is amortised across future migrations rather than charged here.</t>
+          <t>Cost of the migration alone, with the reusable tooling excluded.</t>
         </is>
       </c>
     </row>

</xml_diff>